<commit_message>
deps: openpyxl package version
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3804" yWindow="3540" windowWidth="17280" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -427,7 +427,14 @@
   <dimension ref="B1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="15.88671875" customWidth="1" min="4" max="4"/>
+    <col width="13.109375" bestFit="1" customWidth="1" min="2" max="2"/>
+    <col width="7.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="11" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="6" bestFit="1" customWidth="1" min="5" max="5"/>
+    <col width="2" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="6" bestFit="1" customWidth="1" min="7" max="8"/>
+    <col width="1.5546875" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="1.6640625" bestFit="1" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -488,22 +495,30 @@
           <t>M12345</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>8169326234</v>
-      </c>
-      <c r="E2" t="n">
-        <v>57484</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>TKMOTP12345</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>M12345</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G2" t="n">
-        <v>12345</v>
-      </c>
-      <c r="H2" t="n">
-        <v>87654</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>M12345</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>M12345</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -517,22 +532,30 @@
           <t>M12346</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>8169326235</v>
-      </c>
-      <c r="E3" t="n">
-        <v>57485</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TKMOTP12346</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>M12346</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G3" t="n">
-        <v>12346</v>
-      </c>
-      <c r="H3" t="n">
-        <v>87653</v>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>M12346</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>M12346</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -546,22 +569,30 @@
           <t>M12347</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>8169326236</v>
-      </c>
-      <c r="E4" t="n">
-        <v>57486</v>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TKMOTP12347</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>M12347</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G4" t="n">
-        <v>12347</v>
-      </c>
-      <c r="H4" t="n">
-        <v>87652</v>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>M12347</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>M12347</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -575,22 +606,30 @@
           <t>M12348</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>8169326237</v>
-      </c>
-      <c r="E5" t="n">
-        <v>57487</v>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TKMOTP12348</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>M12348</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G5" t="n">
-        <v>12348</v>
-      </c>
-      <c r="H5" t="n">
-        <v>87651</v>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>M12348</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>M12348</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -604,22 +643,30 @@
           <t>M12349</t>
         </is>
       </c>
-      <c r="D6" t="n">
-        <v>8169326238</v>
-      </c>
-      <c r="E6" t="n">
-        <v>57488</v>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TKMOTP12349</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>M12349</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G6" t="n">
-        <v>12349</v>
-      </c>
-      <c r="H6" t="n">
-        <v>87650</v>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>M12349</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>M12349</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -633,22 +680,30 @@
           <t>M12350</t>
         </is>
       </c>
-      <c r="D7" t="n">
-        <v>8169326239</v>
-      </c>
-      <c r="E7" t="n">
-        <v>57489</v>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>TKMOTP12350</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>M12350</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>12350</v>
-      </c>
-      <c r="H7" t="n">
-        <v>87649</v>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>M12350</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>M12350</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -662,22 +717,30 @@
           <t>M12351</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>8169326240</v>
-      </c>
-      <c r="E8" t="n">
-        <v>57490</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>TKMOTP12351</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>M12351</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G8" t="n">
-        <v>12351</v>
-      </c>
-      <c r="H8" t="n">
-        <v>87648</v>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>M12351</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>M12351</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -691,22 +754,30 @@
           <t>M12352</t>
         </is>
       </c>
-      <c r="D9" t="n">
-        <v>8169326241</v>
-      </c>
-      <c r="E9" t="n">
-        <v>57491</v>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TKMOTP12352</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>M12352</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G9" t="n">
-        <v>12352</v>
-      </c>
-      <c r="H9" t="n">
-        <v>87647</v>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>M12352</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>M12352</t>
+        </is>
       </c>
     </row>
     <row r="10">
@@ -720,22 +791,30 @@
           <t>M12353</t>
         </is>
       </c>
-      <c r="D10" t="n">
-        <v>8169326242</v>
-      </c>
-      <c r="E10" t="n">
-        <v>57492</v>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>TKMOTP12353</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>M12353</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G10" t="n">
-        <v>12353</v>
-      </c>
-      <c r="H10" t="n">
-        <v>87646</v>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>M12353</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>M12353</t>
+        </is>
       </c>
     </row>
     <row r="11">
@@ -749,22 +828,30 @@
           <t>M12354</t>
         </is>
       </c>
-      <c r="D11" t="n">
-        <v>8169326243</v>
-      </c>
-      <c r="E11" t="n">
-        <v>57493</v>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>TKMOTP12354</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>M12354</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G11" t="n">
-        <v>12354</v>
-      </c>
-      <c r="H11" t="n">
-        <v>87645</v>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>M12354</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>M12354</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -778,22 +865,30 @@
           <t>M12355</t>
         </is>
       </c>
-      <c r="D12" t="n">
-        <v>8169326244</v>
-      </c>
-      <c r="E12" t="n">
-        <v>57494</v>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>TKMOTP12355</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>M12355</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G12" t="n">
-        <v>12355</v>
-      </c>
-      <c r="H12" t="n">
-        <v>87644</v>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>M12355</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>M12355</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -807,22 +902,30 @@
           <t>M12356</t>
         </is>
       </c>
-      <c r="D13" t="n">
-        <v>8169326245</v>
-      </c>
-      <c r="E13" t="n">
-        <v>57495</v>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>TKMOTP12356</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>M12356</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G13" t="n">
-        <v>12356</v>
-      </c>
-      <c r="H13" t="n">
-        <v>87643</v>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>M12356</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>M12356</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -836,22 +939,30 @@
           <t>M12357</t>
         </is>
       </c>
-      <c r="D14" t="n">
-        <v>8169326246</v>
-      </c>
-      <c r="E14" t="n">
-        <v>57496</v>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>TKMOTP12357</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>M12357</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G14" t="n">
-        <v>12357</v>
-      </c>
-      <c r="H14" t="n">
-        <v>87642</v>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>M12357</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>M12357</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -865,22 +976,30 @@
           <t>M12358</t>
         </is>
       </c>
-      <c r="D15" t="n">
-        <v>8169326247</v>
-      </c>
-      <c r="E15" t="n">
-        <v>57497</v>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>TKMOTP12358</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>M12358</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>12358</v>
-      </c>
-      <c r="H15" t="n">
-        <v>87641</v>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>M12358</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>M12358</t>
+        </is>
       </c>
     </row>
     <row r="16">
@@ -894,22 +1013,30 @@
           <t>M12359</t>
         </is>
       </c>
-      <c r="D16" t="n">
-        <v>8169326248</v>
-      </c>
-      <c r="E16" t="n">
-        <v>57498</v>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>TKMOTP12359</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>M12359</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>12359</v>
-      </c>
-      <c r="H16" t="n">
-        <v>87640</v>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>M12359</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>M12359</t>
+        </is>
       </c>
     </row>
     <row r="17">
@@ -923,22 +1050,30 @@
           <t>M12360</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>8169326249</v>
-      </c>
-      <c r="E17" t="n">
-        <v>57499</v>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TKMOTP12360</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>M12360</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>12360</v>
-      </c>
-      <c r="H17" t="n">
-        <v>87639</v>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>M12360</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>M12360</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -952,22 +1087,30 @@
           <t>M12361</t>
         </is>
       </c>
-      <c r="D18" t="n">
-        <v>8169326250</v>
-      </c>
-      <c r="E18" t="n">
-        <v>57500</v>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TKMOTP12361</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>M12361</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G18" t="n">
-        <v>12361</v>
-      </c>
-      <c r="H18" t="n">
-        <v>87638</v>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>M12361</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>M12361</t>
+        </is>
       </c>
     </row>
     <row r="19">
@@ -981,22 +1124,30 @@
           <t>M12362</t>
         </is>
       </c>
-      <c r="D19" t="n">
-        <v>8169326251</v>
-      </c>
-      <c r="E19" t="n">
-        <v>57501</v>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>TKMOTP12362</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>M12362</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G19" t="n">
-        <v>12362</v>
-      </c>
-      <c r="H19" t="n">
-        <v>87637</v>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>M12362</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>M12362</t>
+        </is>
       </c>
     </row>
     <row r="20">
@@ -1010,22 +1161,30 @@
           <t>M12363</t>
         </is>
       </c>
-      <c r="D20" t="n">
-        <v>8169326252</v>
-      </c>
-      <c r="E20" t="n">
-        <v>57502</v>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>TKMOTP12363</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>M12363</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G20" t="n">
-        <v>12363</v>
-      </c>
-      <c r="H20" t="n">
-        <v>87636</v>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>M12363</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>M12363</t>
+        </is>
       </c>
     </row>
     <row r="21">
@@ -1039,22 +1198,30 @@
           <t>M12364</t>
         </is>
       </c>
-      <c r="D21" t="n">
-        <v>8169326253</v>
-      </c>
-      <c r="E21" t="n">
-        <v>57503</v>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>TKMOTP12364</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>M12364</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G21" t="n">
-        <v>12364</v>
-      </c>
-      <c r="H21" t="n">
-        <v>87635</v>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>M12364</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>M12364</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -1068,22 +1235,30 @@
           <t>M12365</t>
         </is>
       </c>
-      <c r="D22" t="n">
-        <v>8169326254</v>
-      </c>
-      <c r="E22" t="n">
-        <v>57504</v>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>TKMOTP12365</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>M12365</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G22" t="n">
-        <v>12365</v>
-      </c>
-      <c r="H22" t="n">
-        <v>87634</v>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>M12365</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>M12365</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -1097,22 +1272,30 @@
           <t>M12366</t>
         </is>
       </c>
-      <c r="D23" t="n">
-        <v>8169326255</v>
-      </c>
-      <c r="E23" t="n">
-        <v>57505</v>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>TKMOTP12366</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>M12366</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G23" t="n">
-        <v>12366</v>
-      </c>
-      <c r="H23" t="n">
-        <v>87633</v>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>M12366</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>M12366</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -1126,22 +1309,30 @@
           <t>M12367</t>
         </is>
       </c>
-      <c r="D24" t="n">
-        <v>8169326256</v>
-      </c>
-      <c r="E24" t="n">
-        <v>57506</v>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TKMOTP12367</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>M12367</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G24" t="n">
-        <v>12367</v>
-      </c>
-      <c r="H24" t="n">
-        <v>87632</v>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>M12367</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>M12367</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1155,22 +1346,30 @@
           <t>M12368</t>
         </is>
       </c>
-      <c r="D25" t="n">
-        <v>8169326257</v>
-      </c>
-      <c r="E25" t="n">
-        <v>57507</v>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>TKMOTP12368</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>M12368</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G25" t="n">
-        <v>12368</v>
-      </c>
-      <c r="H25" t="n">
-        <v>87631</v>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>M12368</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>M12368</t>
+        </is>
       </c>
     </row>
     <row r="26">
@@ -1184,22 +1383,30 @@
           <t>M12369</t>
         </is>
       </c>
-      <c r="D26" t="n">
-        <v>8169326258</v>
-      </c>
-      <c r="E26" t="n">
-        <v>57508</v>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>TKMOTP12369</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>M12369</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G26" t="n">
-        <v>12369</v>
-      </c>
-      <c r="H26" t="n">
-        <v>87630</v>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>M12369</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>M12369</t>
+        </is>
       </c>
     </row>
     <row r="27">
@@ -1213,22 +1420,30 @@
           <t>M12370</t>
         </is>
       </c>
-      <c r="D27" t="n">
-        <v>8169326259</v>
-      </c>
-      <c r="E27" t="n">
-        <v>57509</v>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>TKMOTP12370</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>M12370</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G27" t="n">
-        <v>12370</v>
-      </c>
-      <c r="H27" t="n">
-        <v>87629</v>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>M12370</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>M12370</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -1242,22 +1457,30 @@
           <t>M12371</t>
         </is>
       </c>
-      <c r="D28" t="n">
-        <v>8169326260</v>
-      </c>
-      <c r="E28" t="n">
-        <v>57510</v>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>TKMOTP12371</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>M12371</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G28" t="n">
-        <v>12371</v>
-      </c>
-      <c r="H28" t="n">
-        <v>87628</v>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>M12371</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>M12371</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -1271,22 +1494,30 @@
           <t>M12372</t>
         </is>
       </c>
-      <c r="D29" t="n">
-        <v>8169326261</v>
-      </c>
-      <c r="E29" t="n">
-        <v>57511</v>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>TKMOTP12372</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>M12372</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G29" t="n">
-        <v>12372</v>
-      </c>
-      <c r="H29" t="n">
-        <v>87627</v>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>M12372</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>M12372</t>
+        </is>
       </c>
     </row>
     <row r="30">
@@ -1300,22 +1531,30 @@
           <t>M12373</t>
         </is>
       </c>
-      <c r="D30" t="n">
-        <v>8169326262</v>
-      </c>
-      <c r="E30" t="n">
-        <v>57512</v>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>TKMOTP12373</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>M12373</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G30" t="n">
-        <v>12373</v>
-      </c>
-      <c r="H30" t="n">
-        <v>87626</v>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>M12373</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>M12373</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Revert "deps: openpyxl package version"
This reverts commit fcdb83aca9d09fb74813d59d3a5122fd7e5707c7.
</commit_message>
<xml_diff>
--- a/template.xlsx
+++ b/template.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3804" yWindow="3540" windowWidth="17280" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -427,14 +427,7 @@
   <dimension ref="B1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col width="13.109375" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="7.6640625" bestFit="1" customWidth="1" min="3" max="3"/>
-    <col width="11" bestFit="1" customWidth="1" min="4" max="4"/>
-    <col width="6" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="2" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="6" bestFit="1" customWidth="1" min="7" max="8"/>
-    <col width="1.5546875" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="1.6640625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="15.88671875" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -495,30 +488,22 @@
           <t>M12345</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>TKMOTP12345</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>M12345</t>
-        </is>
+      <c r="D2" t="n">
+        <v>8169326234</v>
+      </c>
+      <c r="E2" t="n">
+        <v>57484</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>M12345</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>M12345</t>
-        </is>
+      <c r="G2" t="n">
+        <v>12345</v>
+      </c>
+      <c r="H2" t="n">
+        <v>87654</v>
       </c>
     </row>
     <row r="3">
@@ -532,30 +517,22 @@
           <t>M12346</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>TKMOTP12346</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>M12346</t>
-        </is>
+      <c r="D3" t="n">
+        <v>8169326235</v>
+      </c>
+      <c r="E3" t="n">
+        <v>57485</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>M12346</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>M12346</t>
-        </is>
+      <c r="G3" t="n">
+        <v>12346</v>
+      </c>
+      <c r="H3" t="n">
+        <v>87653</v>
       </c>
     </row>
     <row r="4">
@@ -569,30 +546,22 @@
           <t>M12347</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>TKMOTP12347</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>M12347</t>
-        </is>
+      <c r="D4" t="n">
+        <v>8169326236</v>
+      </c>
+      <c r="E4" t="n">
+        <v>57486</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>M12347</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>M12347</t>
-        </is>
+      <c r="G4" t="n">
+        <v>12347</v>
+      </c>
+      <c r="H4" t="n">
+        <v>87652</v>
       </c>
     </row>
     <row r="5">
@@ -606,30 +575,22 @@
           <t>M12348</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>TKMOTP12348</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>M12348</t>
-        </is>
+      <c r="D5" t="n">
+        <v>8169326237</v>
+      </c>
+      <c r="E5" t="n">
+        <v>57487</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>M12348</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>M12348</t>
-        </is>
+      <c r="G5" t="n">
+        <v>12348</v>
+      </c>
+      <c r="H5" t="n">
+        <v>87651</v>
       </c>
     </row>
     <row r="6">
@@ -643,30 +604,22 @@
           <t>M12349</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>TKMOTP12349</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>M12349</t>
-        </is>
+      <c r="D6" t="n">
+        <v>8169326238</v>
+      </c>
+      <c r="E6" t="n">
+        <v>57488</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>M12349</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>M12349</t>
-        </is>
+      <c r="G6" t="n">
+        <v>12349</v>
+      </c>
+      <c r="H6" t="n">
+        <v>87650</v>
       </c>
     </row>
     <row r="7">
@@ -680,30 +633,22 @@
           <t>M12350</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>TKMOTP12350</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>M12350</t>
-        </is>
+      <c r="D7" t="n">
+        <v>8169326239</v>
+      </c>
+      <c r="E7" t="n">
+        <v>57489</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>M12350</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>M12350</t>
-        </is>
+      <c r="G7" t="n">
+        <v>12350</v>
+      </c>
+      <c r="H7" t="n">
+        <v>87649</v>
       </c>
     </row>
     <row r="8">
@@ -717,30 +662,22 @@
           <t>M12351</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>TKMOTP12351</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>M12351</t>
-        </is>
+      <c r="D8" t="n">
+        <v>8169326240</v>
+      </c>
+      <c r="E8" t="n">
+        <v>57490</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>M12351</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>M12351</t>
-        </is>
+      <c r="G8" t="n">
+        <v>12351</v>
+      </c>
+      <c r="H8" t="n">
+        <v>87648</v>
       </c>
     </row>
     <row r="9">
@@ -754,30 +691,22 @@
           <t>M12352</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>TKMOTP12352</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>M12352</t>
-        </is>
+      <c r="D9" t="n">
+        <v>8169326241</v>
+      </c>
+      <c r="E9" t="n">
+        <v>57491</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>M12352</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>M12352</t>
-        </is>
+      <c r="G9" t="n">
+        <v>12352</v>
+      </c>
+      <c r="H9" t="n">
+        <v>87647</v>
       </c>
     </row>
     <row r="10">
@@ -791,30 +720,22 @@
           <t>M12353</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>TKMOTP12353</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>M12353</t>
-        </is>
+      <c r="D10" t="n">
+        <v>8169326242</v>
+      </c>
+      <c r="E10" t="n">
+        <v>57492</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>M12353</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>M12353</t>
-        </is>
+      <c r="G10" t="n">
+        <v>12353</v>
+      </c>
+      <c r="H10" t="n">
+        <v>87646</v>
       </c>
     </row>
     <row r="11">
@@ -828,30 +749,22 @@
           <t>M12354</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>TKMOTP12354</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>M12354</t>
-        </is>
+      <c r="D11" t="n">
+        <v>8169326243</v>
+      </c>
+      <c r="E11" t="n">
+        <v>57493</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>M12354</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>M12354</t>
-        </is>
+      <c r="G11" t="n">
+        <v>12354</v>
+      </c>
+      <c r="H11" t="n">
+        <v>87645</v>
       </c>
     </row>
     <row r="12">
@@ -865,30 +778,22 @@
           <t>M12355</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>TKMOTP12355</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>M12355</t>
-        </is>
+      <c r="D12" t="n">
+        <v>8169326244</v>
+      </c>
+      <c r="E12" t="n">
+        <v>57494</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>M12355</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>M12355</t>
-        </is>
+      <c r="G12" t="n">
+        <v>12355</v>
+      </c>
+      <c r="H12" t="n">
+        <v>87644</v>
       </c>
     </row>
     <row r="13">
@@ -902,30 +807,22 @@
           <t>M12356</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>TKMOTP12356</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>M12356</t>
-        </is>
+      <c r="D13" t="n">
+        <v>8169326245</v>
+      </c>
+      <c r="E13" t="n">
+        <v>57495</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>M12356</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>M12356</t>
-        </is>
+      <c r="G13" t="n">
+        <v>12356</v>
+      </c>
+      <c r="H13" t="n">
+        <v>87643</v>
       </c>
     </row>
     <row r="14">
@@ -939,30 +836,22 @@
           <t>M12357</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>TKMOTP12357</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>M12357</t>
-        </is>
+      <c r="D14" t="n">
+        <v>8169326246</v>
+      </c>
+      <c r="E14" t="n">
+        <v>57496</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>M12357</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>M12357</t>
-        </is>
+      <c r="G14" t="n">
+        <v>12357</v>
+      </c>
+      <c r="H14" t="n">
+        <v>87642</v>
       </c>
     </row>
     <row r="15">
@@ -976,30 +865,22 @@
           <t>M12358</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>TKMOTP12358</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>M12358</t>
-        </is>
+      <c r="D15" t="n">
+        <v>8169326247</v>
+      </c>
+      <c r="E15" t="n">
+        <v>57497</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>M12358</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>M12358</t>
-        </is>
+      <c r="G15" t="n">
+        <v>12358</v>
+      </c>
+      <c r="H15" t="n">
+        <v>87641</v>
       </c>
     </row>
     <row r="16">
@@ -1013,30 +894,22 @@
           <t>M12359</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>TKMOTP12359</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>M12359</t>
-        </is>
+      <c r="D16" t="n">
+        <v>8169326248</v>
+      </c>
+      <c r="E16" t="n">
+        <v>57498</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>M12359</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>M12359</t>
-        </is>
+      <c r="G16" t="n">
+        <v>12359</v>
+      </c>
+      <c r="H16" t="n">
+        <v>87640</v>
       </c>
     </row>
     <row r="17">
@@ -1050,30 +923,22 @@
           <t>M12360</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>TKMOTP12360</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>M12360</t>
-        </is>
+      <c r="D17" t="n">
+        <v>8169326249</v>
+      </c>
+      <c r="E17" t="n">
+        <v>57499</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>M12360</t>
-        </is>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>M12360</t>
-        </is>
+      <c r="G17" t="n">
+        <v>12360</v>
+      </c>
+      <c r="H17" t="n">
+        <v>87639</v>
       </c>
     </row>
     <row r="18">
@@ -1087,30 +952,22 @@
           <t>M12361</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>TKMOTP12361</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>M12361</t>
-        </is>
+      <c r="D18" t="n">
+        <v>8169326250</v>
+      </c>
+      <c r="E18" t="n">
+        <v>57500</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>M12361</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>M12361</t>
-        </is>
+      <c r="G18" t="n">
+        <v>12361</v>
+      </c>
+      <c r="H18" t="n">
+        <v>87638</v>
       </c>
     </row>
     <row r="19">
@@ -1124,30 +981,22 @@
           <t>M12362</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>TKMOTP12362</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>M12362</t>
-        </is>
+      <c r="D19" t="n">
+        <v>8169326251</v>
+      </c>
+      <c r="E19" t="n">
+        <v>57501</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>M12362</t>
-        </is>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>M12362</t>
-        </is>
+      <c r="G19" t="n">
+        <v>12362</v>
+      </c>
+      <c r="H19" t="n">
+        <v>87637</v>
       </c>
     </row>
     <row r="20">
@@ -1161,30 +1010,22 @@
           <t>M12363</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>TKMOTP12363</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>M12363</t>
-        </is>
+      <c r="D20" t="n">
+        <v>8169326252</v>
+      </c>
+      <c r="E20" t="n">
+        <v>57502</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>M12363</t>
-        </is>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>M12363</t>
-        </is>
+      <c r="G20" t="n">
+        <v>12363</v>
+      </c>
+      <c r="H20" t="n">
+        <v>87636</v>
       </c>
     </row>
     <row r="21">
@@ -1198,30 +1039,22 @@
           <t>M12364</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>TKMOTP12364</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>M12364</t>
-        </is>
+      <c r="D21" t="n">
+        <v>8169326253</v>
+      </c>
+      <c r="E21" t="n">
+        <v>57503</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>M12364</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>M12364</t>
-        </is>
+      <c r="G21" t="n">
+        <v>12364</v>
+      </c>
+      <c r="H21" t="n">
+        <v>87635</v>
       </c>
     </row>
     <row r="22">
@@ -1235,30 +1068,22 @@
           <t>M12365</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>TKMOTP12365</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>M12365</t>
-        </is>
+      <c r="D22" t="n">
+        <v>8169326254</v>
+      </c>
+      <c r="E22" t="n">
+        <v>57504</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>M12365</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>M12365</t>
-        </is>
+      <c r="G22" t="n">
+        <v>12365</v>
+      </c>
+      <c r="H22" t="n">
+        <v>87634</v>
       </c>
     </row>
     <row r="23">
@@ -1272,30 +1097,22 @@
           <t>M12366</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>TKMOTP12366</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>M12366</t>
-        </is>
+      <c r="D23" t="n">
+        <v>8169326255</v>
+      </c>
+      <c r="E23" t="n">
+        <v>57505</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>M12366</t>
-        </is>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>M12366</t>
-        </is>
+      <c r="G23" t="n">
+        <v>12366</v>
+      </c>
+      <c r="H23" t="n">
+        <v>87633</v>
       </c>
     </row>
     <row r="24">
@@ -1309,30 +1126,22 @@
           <t>M12367</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>TKMOTP12367</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>M12367</t>
-        </is>
+      <c r="D24" t="n">
+        <v>8169326256</v>
+      </c>
+      <c r="E24" t="n">
+        <v>57506</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>M12367</t>
-        </is>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>M12367</t>
-        </is>
+      <c r="G24" t="n">
+        <v>12367</v>
+      </c>
+      <c r="H24" t="n">
+        <v>87632</v>
       </c>
     </row>
     <row r="25">
@@ -1346,30 +1155,22 @@
           <t>M12368</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>TKMOTP12368</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>M12368</t>
-        </is>
+      <c r="D25" t="n">
+        <v>8169326257</v>
+      </c>
+      <c r="E25" t="n">
+        <v>57507</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>M12368</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>M12368</t>
-        </is>
+      <c r="G25" t="n">
+        <v>12368</v>
+      </c>
+      <c r="H25" t="n">
+        <v>87631</v>
       </c>
     </row>
     <row r="26">
@@ -1383,30 +1184,22 @@
           <t>M12369</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>TKMOTP12369</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>M12369</t>
-        </is>
+      <c r="D26" t="n">
+        <v>8169326258</v>
+      </c>
+      <c r="E26" t="n">
+        <v>57508</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>M12369</t>
-        </is>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>M12369</t>
-        </is>
+      <c r="G26" t="n">
+        <v>12369</v>
+      </c>
+      <c r="H26" t="n">
+        <v>87630</v>
       </c>
     </row>
     <row r="27">
@@ -1420,30 +1213,22 @@
           <t>M12370</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>TKMOTP12370</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>M12370</t>
-        </is>
+      <c r="D27" t="n">
+        <v>8169326259</v>
+      </c>
+      <c r="E27" t="n">
+        <v>57509</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>M12370</t>
-        </is>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>M12370</t>
-        </is>
+      <c r="G27" t="n">
+        <v>12370</v>
+      </c>
+      <c r="H27" t="n">
+        <v>87629</v>
       </c>
     </row>
     <row r="28">
@@ -1457,30 +1242,22 @@
           <t>M12371</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>TKMOTP12371</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>M12371</t>
-        </is>
+      <c r="D28" t="n">
+        <v>8169326260</v>
+      </c>
+      <c r="E28" t="n">
+        <v>57510</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>M12371</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>M12371</t>
-        </is>
+      <c r="G28" t="n">
+        <v>12371</v>
+      </c>
+      <c r="H28" t="n">
+        <v>87628</v>
       </c>
     </row>
     <row r="29">
@@ -1494,30 +1271,22 @@
           <t>M12372</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>TKMOTP12372</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>M12372</t>
-        </is>
+      <c r="D29" t="n">
+        <v>8169326261</v>
+      </c>
+      <c r="E29" t="n">
+        <v>57511</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>M12372</t>
-        </is>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>M12372</t>
-        </is>
+      <c r="G29" t="n">
+        <v>12372</v>
+      </c>
+      <c r="H29" t="n">
+        <v>87627</v>
       </c>
     </row>
     <row r="30">
@@ -1531,30 +1300,22 @@
           <t>M12373</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>TKMOTP12373</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>M12373</t>
-        </is>
+      <c r="D30" t="n">
+        <v>8169326262</v>
+      </c>
+      <c r="E30" t="n">
+        <v>57512</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>M12373</t>
-        </is>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>M12373</t>
-        </is>
+      <c r="G30" t="n">
+        <v>12373</v>
+      </c>
+      <c r="H30" t="n">
+        <v>87626</v>
       </c>
     </row>
   </sheetData>

</xml_diff>